<commit_message>
Ship company-document memos, payslip email, and People360 1.0.3.
Timekeeping memos now email a legal PDF that matches Memo Preview field size and layout, and this release also includes the form builder, payslip sending, and related payroll/employee updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_upload_template.xlsx
+++ b/resources/templates/employee_upload_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="301">
   <si>
     <t>employee_number</t>
   </si>
@@ -77,6 +77,15 @@
     <t>tax_status</t>
   </si>
   <si>
+    <t>bank_name</t>
+  </si>
+  <si>
+    <t>bank_account_number</t>
+  </si>
+  <si>
+    <t>bank_account_type</t>
+  </si>
+  <si>
     <t>campus_code</t>
   </si>
   <si>
@@ -482,6 +491,15 @@
     <t>Tax Status</t>
   </si>
   <si>
+    <t>Bank Name</t>
+  </si>
+  <si>
+    <t>Account Number</t>
+  </si>
+  <si>
+    <t>Account Type (savings/checking/payroll)</t>
+  </si>
+  <si>
     <t>Campus Code</t>
   </si>
   <si>
@@ -837,6 +855,15 @@
   </si>
   <si>
     <t>Dela Cruz</t>
+  </si>
+  <si>
+    <t>BDO</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>savings</t>
   </si>
   <si>
     <t>AG</t>
@@ -1231,10 +1258,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:EE154"/>
+  <dimension ref="A1:EH154"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:135">
+    <row r="1" spans="1:138">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1640,486 +1667,513 @@
       <c r="EE1" t="s">
         <v>134</v>
       </c>
+      <c r="EF1" t="s">
+        <v>135</v>
+      </c>
+      <c r="EG1" t="s">
+        <v>136</v>
+      </c>
+      <c r="EH1" t="s">
+        <v>137</v>
+      </c>
     </row>
-    <row r="2" spans="1:135">
+    <row r="2" spans="1:138">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="G2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="H2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="K2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="L2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="M2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="O2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="P2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="Q2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="R2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="S2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="T2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="U2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="V2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="W2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="X2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="Y2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="Z2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="AB2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="AC2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="AD2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="AE2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="AF2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="AG2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="AH2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="AI2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AJ2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AK2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AL2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AM2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="AN2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="AO2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AP2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AQ2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AR2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AS2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AT2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="AU2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="AV2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="AW2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AX2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AY2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="AZ2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="BA2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="BB2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="BC2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="BD2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="BE2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="BF2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="BG2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="BH2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="BI2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="BJ2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="BK2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="BL2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="BM2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="BN2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="BO2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="BP2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="BQ2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="BR2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="BS2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="BT2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="BU2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="BV2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="BW2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="BX2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="BY2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="BZ2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="CA2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="CB2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="CC2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="CD2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="CE2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="CF2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="CG2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="CH2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="CI2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="CJ2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="CK2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="CL2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="CM2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="CN2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="CO2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="CP2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="CQ2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="CR2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="CS2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="CT2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="CU2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="CV2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="CW2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="CX2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="CY2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="CZ2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="DA2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="DB2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="DC2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="DD2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="DE2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="DF2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="DG2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="DH2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="DI2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="DJ2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="DK2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="DL2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="DM2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="DN2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="DO2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="DP2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="DQ2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="DR2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="DS2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="DT2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="DU2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="DV2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="DW2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="DX2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="DY2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="DZ2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="EA2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="EB2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="EC2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="ED2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="EE2" t="s">
-        <v>269</v>
+        <v>272</v>
+      </c>
+      <c r="EF2" t="s">
+        <v>273</v>
+      </c>
+      <c r="EG2" t="s">
+        <v>274</v>
+      </c>
+      <c r="EH2" t="s">
+        <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:135">
+    <row r="3" spans="1:138">
       <c r="A3" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B3" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C3" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="U3" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="V3" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="W3" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="X3" t="s">
-        <v>276</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>277</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>278</v>
-      </c>
-      <c r="AV3" t="s">
-        <v>279</v>
+        <v>283</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>284</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>285</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>285</v>
       </c>
       <c r="AW3" t="s">
-        <v>280</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>281</v>
-      </c>
-      <c r="BJ3" t="s">
-        <v>282</v>
+        <v>286</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>287</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>288</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>289</v>
       </c>
       <c r="BK3" t="s">
-        <v>283</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>284</v>
+        <v>290</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>291</v>
+      </c>
+      <c r="BN3" t="s">
+        <v>292</v>
       </c>
       <c r="BO3" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="BR3" t="s">
-        <v>286</v>
-      </c>
-      <c r="CJ3" t="s">
-        <v>287</v>
-      </c>
-      <c r="CK3" t="s">
-        <v>288</v>
-      </c>
-      <c r="CT3" t="s">
-        <v>289</v>
-      </c>
-      <c r="DA3" t="s">
-        <v>290</v>
-      </c>
-      <c r="DC3" t="s">
-        <v>291</v>
+        <v>294</v>
+      </c>
+      <c r="BU3" t="s">
+        <v>295</v>
+      </c>
+      <c r="CM3" t="s">
+        <v>296</v>
+      </c>
+      <c r="CN3" t="s">
+        <v>297</v>
+      </c>
+      <c r="CW3" t="s">
+        <v>298</v>
+      </c>
+      <c r="DD3" t="s">
+        <v>299</v>
+      </c>
+      <c r="DF3" t="s">
+        <v>300</v>
       </c>
     </row>
-    <row r="4" spans="1:135">
+    <row r="4" spans="1:138">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -2255,8 +2309,11 @@
       <c r="EC4" s="1"/>
       <c r="ED4" s="1"/>
       <c r="EE4" s="1"/>
+      <c r="EF4" s="1"/>
+      <c r="EG4" s="1"/>
+      <c r="EH4" s="1"/>
     </row>
-    <row r="5" spans="1:135">
+    <row r="5" spans="1:138">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -2392,8 +2449,11 @@
       <c r="EC5" s="1"/>
       <c r="ED5" s="1"/>
       <c r="EE5" s="1"/>
+      <c r="EF5" s="1"/>
+      <c r="EG5" s="1"/>
+      <c r="EH5" s="1"/>
     </row>
-    <row r="6" spans="1:135">
+    <row r="6" spans="1:138">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -2529,8 +2589,11 @@
       <c r="EC6" s="1"/>
       <c r="ED6" s="1"/>
       <c r="EE6" s="1"/>
+      <c r="EF6" s="1"/>
+      <c r="EG6" s="1"/>
+      <c r="EH6" s="1"/>
     </row>
-    <row r="7" spans="1:135">
+    <row r="7" spans="1:138">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2666,8 +2729,11 @@
       <c r="EC7" s="1"/>
       <c r="ED7" s="1"/>
       <c r="EE7" s="1"/>
+      <c r="EF7" s="1"/>
+      <c r="EG7" s="1"/>
+      <c r="EH7" s="1"/>
     </row>
-    <row r="8" spans="1:135">
+    <row r="8" spans="1:138">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -2803,8 +2869,11 @@
       <c r="EC8" s="1"/>
       <c r="ED8" s="1"/>
       <c r="EE8" s="1"/>
+      <c r="EF8" s="1"/>
+      <c r="EG8" s="1"/>
+      <c r="EH8" s="1"/>
     </row>
-    <row r="9" spans="1:135">
+    <row r="9" spans="1:138">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -2940,8 +3009,11 @@
       <c r="EC9" s="1"/>
       <c r="ED9" s="1"/>
       <c r="EE9" s="1"/>
+      <c r="EF9" s="1"/>
+      <c r="EG9" s="1"/>
+      <c r="EH9" s="1"/>
     </row>
-    <row r="10" spans="1:135">
+    <row r="10" spans="1:138">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -3077,8 +3149,11 @@
       <c r="EC10" s="1"/>
       <c r="ED10" s="1"/>
       <c r="EE10" s="1"/>
+      <c r="EF10" s="1"/>
+      <c r="EG10" s="1"/>
+      <c r="EH10" s="1"/>
     </row>
-    <row r="11" spans="1:135">
+    <row r="11" spans="1:138">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -3214,8 +3289,11 @@
       <c r="EC11" s="1"/>
       <c r="ED11" s="1"/>
       <c r="EE11" s="1"/>
+      <c r="EF11" s="1"/>
+      <c r="EG11" s="1"/>
+      <c r="EH11" s="1"/>
     </row>
-    <row r="12" spans="1:135">
+    <row r="12" spans="1:138">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -3351,8 +3429,11 @@
       <c r="EC12" s="1"/>
       <c r="ED12" s="1"/>
       <c r="EE12" s="1"/>
+      <c r="EF12" s="1"/>
+      <c r="EG12" s="1"/>
+      <c r="EH12" s="1"/>
     </row>
-    <row r="13" spans="1:135">
+    <row r="13" spans="1:138">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -3488,8 +3569,11 @@
       <c r="EC13" s="1"/>
       <c r="ED13" s="1"/>
       <c r="EE13" s="1"/>
+      <c r="EF13" s="1"/>
+      <c r="EG13" s="1"/>
+      <c r="EH13" s="1"/>
     </row>
-    <row r="14" spans="1:135">
+    <row r="14" spans="1:138">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -3625,8 +3709,11 @@
       <c r="EC14" s="1"/>
       <c r="ED14" s="1"/>
       <c r="EE14" s="1"/>
+      <c r="EF14" s="1"/>
+      <c r="EG14" s="1"/>
+      <c r="EH14" s="1"/>
     </row>
-    <row r="15" spans="1:135">
+    <row r="15" spans="1:138">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -3762,8 +3849,11 @@
       <c r="EC15" s="1"/>
       <c r="ED15" s="1"/>
       <c r="EE15" s="1"/>
+      <c r="EF15" s="1"/>
+      <c r="EG15" s="1"/>
+      <c r="EH15" s="1"/>
     </row>
-    <row r="16" spans="1:135">
+    <row r="16" spans="1:138">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -3899,8 +3989,11 @@
       <c r="EC16" s="1"/>
       <c r="ED16" s="1"/>
       <c r="EE16" s="1"/>
+      <c r="EF16" s="1"/>
+      <c r="EG16" s="1"/>
+      <c r="EH16" s="1"/>
     </row>
-    <row r="17" spans="1:135">
+    <row r="17" spans="1:138">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -4036,8 +4129,11 @@
       <c r="EC17" s="1"/>
       <c r="ED17" s="1"/>
       <c r="EE17" s="1"/>
+      <c r="EF17" s="1"/>
+      <c r="EG17" s="1"/>
+      <c r="EH17" s="1"/>
     </row>
-    <row r="18" spans="1:135">
+    <row r="18" spans="1:138">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -4173,8 +4269,11 @@
       <c r="EC18" s="1"/>
       <c r="ED18" s="1"/>
       <c r="EE18" s="1"/>
+      <c r="EF18" s="1"/>
+      <c r="EG18" s="1"/>
+      <c r="EH18" s="1"/>
     </row>
-    <row r="19" spans="1:135">
+    <row r="19" spans="1:138">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -4310,8 +4409,11 @@
       <c r="EC19" s="1"/>
       <c r="ED19" s="1"/>
       <c r="EE19" s="1"/>
+      <c r="EF19" s="1"/>
+      <c r="EG19" s="1"/>
+      <c r="EH19" s="1"/>
     </row>
-    <row r="20" spans="1:135">
+    <row r="20" spans="1:138">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -4447,8 +4549,11 @@
       <c r="EC20" s="1"/>
       <c r="ED20" s="1"/>
       <c r="EE20" s="1"/>
+      <c r="EF20" s="1"/>
+      <c r="EG20" s="1"/>
+      <c r="EH20" s="1"/>
     </row>
-    <row r="21" spans="1:135">
+    <row r="21" spans="1:138">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -4584,8 +4689,11 @@
       <c r="EC21" s="1"/>
       <c r="ED21" s="1"/>
       <c r="EE21" s="1"/>
+      <c r="EF21" s="1"/>
+      <c r="EG21" s="1"/>
+      <c r="EH21" s="1"/>
     </row>
-    <row r="22" spans="1:135">
+    <row r="22" spans="1:138">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -4721,8 +4829,11 @@
       <c r="EC22" s="1"/>
       <c r="ED22" s="1"/>
       <c r="EE22" s="1"/>
+      <c r="EF22" s="1"/>
+      <c r="EG22" s="1"/>
+      <c r="EH22" s="1"/>
     </row>
-    <row r="23" spans="1:135">
+    <row r="23" spans="1:138">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -4858,8 +4969,11 @@
       <c r="EC23" s="1"/>
       <c r="ED23" s="1"/>
       <c r="EE23" s="1"/>
+      <c r="EF23" s="1"/>
+      <c r="EG23" s="1"/>
+      <c r="EH23" s="1"/>
     </row>
-    <row r="24" spans="1:135">
+    <row r="24" spans="1:138">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -4995,8 +5109,11 @@
       <c r="EC24" s="1"/>
       <c r="ED24" s="1"/>
       <c r="EE24" s="1"/>
+      <c r="EF24" s="1"/>
+      <c r="EG24" s="1"/>
+      <c r="EH24" s="1"/>
     </row>
-    <row r="25" spans="1:135">
+    <row r="25" spans="1:138">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -5132,8 +5249,11 @@
       <c r="EC25" s="1"/>
       <c r="ED25" s="1"/>
       <c r="EE25" s="1"/>
+      <c r="EF25" s="1"/>
+      <c r="EG25" s="1"/>
+      <c r="EH25" s="1"/>
     </row>
-    <row r="26" spans="1:135">
+    <row r="26" spans="1:138">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -5269,8 +5389,11 @@
       <c r="EC26" s="1"/>
       <c r="ED26" s="1"/>
       <c r="EE26" s="1"/>
+      <c r="EF26" s="1"/>
+      <c r="EG26" s="1"/>
+      <c r="EH26" s="1"/>
     </row>
-    <row r="27" spans="1:135">
+    <row r="27" spans="1:138">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -5406,8 +5529,11 @@
       <c r="EC27" s="1"/>
       <c r="ED27" s="1"/>
       <c r="EE27" s="1"/>
+      <c r="EF27" s="1"/>
+      <c r="EG27" s="1"/>
+      <c r="EH27" s="1"/>
     </row>
-    <row r="28" spans="1:135">
+    <row r="28" spans="1:138">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -5543,8 +5669,11 @@
       <c r="EC28" s="1"/>
       <c r="ED28" s="1"/>
       <c r="EE28" s="1"/>
+      <c r="EF28" s="1"/>
+      <c r="EG28" s="1"/>
+      <c r="EH28" s="1"/>
     </row>
-    <row r="29" spans="1:135">
+    <row r="29" spans="1:138">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -5680,8 +5809,11 @@
       <c r="EC29" s="1"/>
       <c r="ED29" s="1"/>
       <c r="EE29" s="1"/>
+      <c r="EF29" s="1"/>
+      <c r="EG29" s="1"/>
+      <c r="EH29" s="1"/>
     </row>
-    <row r="30" spans="1:135">
+    <row r="30" spans="1:138">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -5817,8 +5949,11 @@
       <c r="EC30" s="1"/>
       <c r="ED30" s="1"/>
       <c r="EE30" s="1"/>
+      <c r="EF30" s="1"/>
+      <c r="EG30" s="1"/>
+      <c r="EH30" s="1"/>
     </row>
-    <row r="31" spans="1:135">
+    <row r="31" spans="1:138">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -5954,8 +6089,11 @@
       <c r="EC31" s="1"/>
       <c r="ED31" s="1"/>
       <c r="EE31" s="1"/>
+      <c r="EF31" s="1"/>
+      <c r="EG31" s="1"/>
+      <c r="EH31" s="1"/>
     </row>
-    <row r="32" spans="1:135">
+    <row r="32" spans="1:138">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -6091,8 +6229,11 @@
       <c r="EC32" s="1"/>
       <c r="ED32" s="1"/>
       <c r="EE32" s="1"/>
+      <c r="EF32" s="1"/>
+      <c r="EG32" s="1"/>
+      <c r="EH32" s="1"/>
     </row>
-    <row r="33" spans="1:135">
+    <row r="33" spans="1:138">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -6228,8 +6369,11 @@
       <c r="EC33" s="1"/>
       <c r="ED33" s="1"/>
       <c r="EE33" s="1"/>
+      <c r="EF33" s="1"/>
+      <c r="EG33" s="1"/>
+      <c r="EH33" s="1"/>
     </row>
-    <row r="34" spans="1:135">
+    <row r="34" spans="1:138">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -6365,8 +6509,11 @@
       <c r="EC34" s="1"/>
       <c r="ED34" s="1"/>
       <c r="EE34" s="1"/>
+      <c r="EF34" s="1"/>
+      <c r="EG34" s="1"/>
+      <c r="EH34" s="1"/>
     </row>
-    <row r="35" spans="1:135">
+    <row r="35" spans="1:138">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -6502,8 +6649,11 @@
       <c r="EC35" s="1"/>
       <c r="ED35" s="1"/>
       <c r="EE35" s="1"/>
+      <c r="EF35" s="1"/>
+      <c r="EG35" s="1"/>
+      <c r="EH35" s="1"/>
     </row>
-    <row r="36" spans="1:135">
+    <row r="36" spans="1:138">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -6639,8 +6789,11 @@
       <c r="EC36" s="1"/>
       <c r="ED36" s="1"/>
       <c r="EE36" s="1"/>
+      <c r="EF36" s="1"/>
+      <c r="EG36" s="1"/>
+      <c r="EH36" s="1"/>
     </row>
-    <row r="37" spans="1:135">
+    <row r="37" spans="1:138">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -6776,8 +6929,11 @@
       <c r="EC37" s="1"/>
       <c r="ED37" s="1"/>
       <c r="EE37" s="1"/>
+      <c r="EF37" s="1"/>
+      <c r="EG37" s="1"/>
+      <c r="EH37" s="1"/>
     </row>
-    <row r="38" spans="1:135">
+    <row r="38" spans="1:138">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -6913,8 +7069,11 @@
       <c r="EC38" s="1"/>
       <c r="ED38" s="1"/>
       <c r="EE38" s="1"/>
+      <c r="EF38" s="1"/>
+      <c r="EG38" s="1"/>
+      <c r="EH38" s="1"/>
     </row>
-    <row r="39" spans="1:135">
+    <row r="39" spans="1:138">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -7050,8 +7209,11 @@
       <c r="EC39" s="1"/>
       <c r="ED39" s="1"/>
       <c r="EE39" s="1"/>
+      <c r="EF39" s="1"/>
+      <c r="EG39" s="1"/>
+      <c r="EH39" s="1"/>
     </row>
-    <row r="40" spans="1:135">
+    <row r="40" spans="1:138">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -7187,8 +7349,11 @@
       <c r="EC40" s="1"/>
       <c r="ED40" s="1"/>
       <c r="EE40" s="1"/>
+      <c r="EF40" s="1"/>
+      <c r="EG40" s="1"/>
+      <c r="EH40" s="1"/>
     </row>
-    <row r="41" spans="1:135">
+    <row r="41" spans="1:138">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -7324,8 +7489,11 @@
       <c r="EC41" s="1"/>
       <c r="ED41" s="1"/>
       <c r="EE41" s="1"/>
+      <c r="EF41" s="1"/>
+      <c r="EG41" s="1"/>
+      <c r="EH41" s="1"/>
     </row>
-    <row r="42" spans="1:135">
+    <row r="42" spans="1:138">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -7461,8 +7629,11 @@
       <c r="EC42" s="1"/>
       <c r="ED42" s="1"/>
       <c r="EE42" s="1"/>
+      <c r="EF42" s="1"/>
+      <c r="EG42" s="1"/>
+      <c r="EH42" s="1"/>
     </row>
-    <row r="43" spans="1:135">
+    <row r="43" spans="1:138">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -7598,8 +7769,11 @@
       <c r="EC43" s="1"/>
       <c r="ED43" s="1"/>
       <c r="EE43" s="1"/>
+      <c r="EF43" s="1"/>
+      <c r="EG43" s="1"/>
+      <c r="EH43" s="1"/>
     </row>
-    <row r="44" spans="1:135">
+    <row r="44" spans="1:138">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -7735,8 +7909,11 @@
       <c r="EC44" s="1"/>
       <c r="ED44" s="1"/>
       <c r="EE44" s="1"/>
+      <c r="EF44" s="1"/>
+      <c r="EG44" s="1"/>
+      <c r="EH44" s="1"/>
     </row>
-    <row r="45" spans="1:135">
+    <row r="45" spans="1:138">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -7872,8 +8049,11 @@
       <c r="EC45" s="1"/>
       <c r="ED45" s="1"/>
       <c r="EE45" s="1"/>
+      <c r="EF45" s="1"/>
+      <c r="EG45" s="1"/>
+      <c r="EH45" s="1"/>
     </row>
-    <row r="46" spans="1:135">
+    <row r="46" spans="1:138">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -8009,8 +8189,11 @@
       <c r="EC46" s="1"/>
       <c r="ED46" s="1"/>
       <c r="EE46" s="1"/>
+      <c r="EF46" s="1"/>
+      <c r="EG46" s="1"/>
+      <c r="EH46" s="1"/>
     </row>
-    <row r="47" spans="1:135">
+    <row r="47" spans="1:138">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -8146,8 +8329,11 @@
       <c r="EC47" s="1"/>
       <c r="ED47" s="1"/>
       <c r="EE47" s="1"/>
+      <c r="EF47" s="1"/>
+      <c r="EG47" s="1"/>
+      <c r="EH47" s="1"/>
     </row>
-    <row r="48" spans="1:135">
+    <row r="48" spans="1:138">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -8283,8 +8469,11 @@
       <c r="EC48" s="1"/>
       <c r="ED48" s="1"/>
       <c r="EE48" s="1"/>
+      <c r="EF48" s="1"/>
+      <c r="EG48" s="1"/>
+      <c r="EH48" s="1"/>
     </row>
-    <row r="49" spans="1:135">
+    <row r="49" spans="1:138">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -8420,8 +8609,11 @@
       <c r="EC49" s="1"/>
       <c r="ED49" s="1"/>
       <c r="EE49" s="1"/>
+      <c r="EF49" s="1"/>
+      <c r="EG49" s="1"/>
+      <c r="EH49" s="1"/>
     </row>
-    <row r="50" spans="1:135">
+    <row r="50" spans="1:138">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -8557,8 +8749,11 @@
       <c r="EC50" s="1"/>
       <c r="ED50" s="1"/>
       <c r="EE50" s="1"/>
+      <c r="EF50" s="1"/>
+      <c r="EG50" s="1"/>
+      <c r="EH50" s="1"/>
     </row>
-    <row r="51" spans="1:135">
+    <row r="51" spans="1:138">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -8694,8 +8889,11 @@
       <c r="EC51" s="1"/>
       <c r="ED51" s="1"/>
       <c r="EE51" s="1"/>
+      <c r="EF51" s="1"/>
+      <c r="EG51" s="1"/>
+      <c r="EH51" s="1"/>
     </row>
-    <row r="52" spans="1:135">
+    <row r="52" spans="1:138">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -8831,8 +9029,11 @@
       <c r="EC52" s="1"/>
       <c r="ED52" s="1"/>
       <c r="EE52" s="1"/>
+      <c r="EF52" s="1"/>
+      <c r="EG52" s="1"/>
+      <c r="EH52" s="1"/>
     </row>
-    <row r="53" spans="1:135">
+    <row r="53" spans="1:138">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -8968,8 +9169,11 @@
       <c r="EC53" s="1"/>
       <c r="ED53" s="1"/>
       <c r="EE53" s="1"/>
+      <c r="EF53" s="1"/>
+      <c r="EG53" s="1"/>
+      <c r="EH53" s="1"/>
     </row>
-    <row r="54" spans="1:135">
+    <row r="54" spans="1:138">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -9105,8 +9309,11 @@
       <c r="EC54" s="1"/>
       <c r="ED54" s="1"/>
       <c r="EE54" s="1"/>
+      <c r="EF54" s="1"/>
+      <c r="EG54" s="1"/>
+      <c r="EH54" s="1"/>
     </row>
-    <row r="55" spans="1:135">
+    <row r="55" spans="1:138">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -9242,8 +9449,11 @@
       <c r="EC55" s="1"/>
       <c r="ED55" s="1"/>
       <c r="EE55" s="1"/>
+      <c r="EF55" s="1"/>
+      <c r="EG55" s="1"/>
+      <c r="EH55" s="1"/>
     </row>
-    <row r="56" spans="1:135">
+    <row r="56" spans="1:138">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -9379,8 +9589,11 @@
       <c r="EC56" s="1"/>
       <c r="ED56" s="1"/>
       <c r="EE56" s="1"/>
+      <c r="EF56" s="1"/>
+      <c r="EG56" s="1"/>
+      <c r="EH56" s="1"/>
     </row>
-    <row r="57" spans="1:135">
+    <row r="57" spans="1:138">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -9516,8 +9729,11 @@
       <c r="EC57" s="1"/>
       <c r="ED57" s="1"/>
       <c r="EE57" s="1"/>
+      <c r="EF57" s="1"/>
+      <c r="EG57" s="1"/>
+      <c r="EH57" s="1"/>
     </row>
-    <row r="58" spans="1:135">
+    <row r="58" spans="1:138">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -9653,8 +9869,11 @@
       <c r="EC58" s="1"/>
       <c r="ED58" s="1"/>
       <c r="EE58" s="1"/>
+      <c r="EF58" s="1"/>
+      <c r="EG58" s="1"/>
+      <c r="EH58" s="1"/>
     </row>
-    <row r="59" spans="1:135">
+    <row r="59" spans="1:138">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -9790,8 +10009,11 @@
       <c r="EC59" s="1"/>
       <c r="ED59" s="1"/>
       <c r="EE59" s="1"/>
+      <c r="EF59" s="1"/>
+      <c r="EG59" s="1"/>
+      <c r="EH59" s="1"/>
     </row>
-    <row r="60" spans="1:135">
+    <row r="60" spans="1:138">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -9927,8 +10149,11 @@
       <c r="EC60" s="1"/>
       <c r="ED60" s="1"/>
       <c r="EE60" s="1"/>
+      <c r="EF60" s="1"/>
+      <c r="EG60" s="1"/>
+      <c r="EH60" s="1"/>
     </row>
-    <row r="61" spans="1:135">
+    <row r="61" spans="1:138">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -10064,8 +10289,11 @@
       <c r="EC61" s="1"/>
       <c r="ED61" s="1"/>
       <c r="EE61" s="1"/>
+      <c r="EF61" s="1"/>
+      <c r="EG61" s="1"/>
+      <c r="EH61" s="1"/>
     </row>
-    <row r="62" spans="1:135">
+    <row r="62" spans="1:138">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -10201,8 +10429,11 @@
       <c r="EC62" s="1"/>
       <c r="ED62" s="1"/>
       <c r="EE62" s="1"/>
+      <c r="EF62" s="1"/>
+      <c r="EG62" s="1"/>
+      <c r="EH62" s="1"/>
     </row>
-    <row r="63" spans="1:135">
+    <row r="63" spans="1:138">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -10338,8 +10569,11 @@
       <c r="EC63" s="1"/>
       <c r="ED63" s="1"/>
       <c r="EE63" s="1"/>
+      <c r="EF63" s="1"/>
+      <c r="EG63" s="1"/>
+      <c r="EH63" s="1"/>
     </row>
-    <row r="64" spans="1:135">
+    <row r="64" spans="1:138">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -10475,8 +10709,11 @@
       <c r="EC64" s="1"/>
       <c r="ED64" s="1"/>
       <c r="EE64" s="1"/>
+      <c r="EF64" s="1"/>
+      <c r="EG64" s="1"/>
+      <c r="EH64" s="1"/>
     </row>
-    <row r="65" spans="1:135">
+    <row r="65" spans="1:138">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -10612,8 +10849,11 @@
       <c r="EC65" s="1"/>
       <c r="ED65" s="1"/>
       <c r="EE65" s="1"/>
+      <c r="EF65" s="1"/>
+      <c r="EG65" s="1"/>
+      <c r="EH65" s="1"/>
     </row>
-    <row r="66" spans="1:135">
+    <row r="66" spans="1:138">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -10749,8 +10989,11 @@
       <c r="EC66" s="1"/>
       <c r="ED66" s="1"/>
       <c r="EE66" s="1"/>
+      <c r="EF66" s="1"/>
+      <c r="EG66" s="1"/>
+      <c r="EH66" s="1"/>
     </row>
-    <row r="67" spans="1:135">
+    <row r="67" spans="1:138">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -10886,8 +11129,11 @@
       <c r="EC67" s="1"/>
       <c r="ED67" s="1"/>
       <c r="EE67" s="1"/>
+      <c r="EF67" s="1"/>
+      <c r="EG67" s="1"/>
+      <c r="EH67" s="1"/>
     </row>
-    <row r="68" spans="1:135">
+    <row r="68" spans="1:138">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -11023,8 +11269,11 @@
       <c r="EC68" s="1"/>
       <c r="ED68" s="1"/>
       <c r="EE68" s="1"/>
+      <c r="EF68" s="1"/>
+      <c r="EG68" s="1"/>
+      <c r="EH68" s="1"/>
     </row>
-    <row r="69" spans="1:135">
+    <row r="69" spans="1:138">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -11160,8 +11409,11 @@
       <c r="EC69" s="1"/>
       <c r="ED69" s="1"/>
       <c r="EE69" s="1"/>
+      <c r="EF69" s="1"/>
+      <c r="EG69" s="1"/>
+      <c r="EH69" s="1"/>
     </row>
-    <row r="70" spans="1:135">
+    <row r="70" spans="1:138">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -11297,8 +11549,11 @@
       <c r="EC70" s="1"/>
       <c r="ED70" s="1"/>
       <c r="EE70" s="1"/>
+      <c r="EF70" s="1"/>
+      <c r="EG70" s="1"/>
+      <c r="EH70" s="1"/>
     </row>
-    <row r="71" spans="1:135">
+    <row r="71" spans="1:138">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -11434,8 +11689,11 @@
       <c r="EC71" s="1"/>
       <c r="ED71" s="1"/>
       <c r="EE71" s="1"/>
+      <c r="EF71" s="1"/>
+      <c r="EG71" s="1"/>
+      <c r="EH71" s="1"/>
     </row>
-    <row r="72" spans="1:135">
+    <row r="72" spans="1:138">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -11571,8 +11829,11 @@
       <c r="EC72" s="1"/>
       <c r="ED72" s="1"/>
       <c r="EE72" s="1"/>
+      <c r="EF72" s="1"/>
+      <c r="EG72" s="1"/>
+      <c r="EH72" s="1"/>
     </row>
-    <row r="73" spans="1:135">
+    <row r="73" spans="1:138">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -11708,8 +11969,11 @@
       <c r="EC73" s="1"/>
       <c r="ED73" s="1"/>
       <c r="EE73" s="1"/>
+      <c r="EF73" s="1"/>
+      <c r="EG73" s="1"/>
+      <c r="EH73" s="1"/>
     </row>
-    <row r="74" spans="1:135">
+    <row r="74" spans="1:138">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -11845,8 +12109,11 @@
       <c r="EC74" s="1"/>
       <c r="ED74" s="1"/>
       <c r="EE74" s="1"/>
+      <c r="EF74" s="1"/>
+      <c r="EG74" s="1"/>
+      <c r="EH74" s="1"/>
     </row>
-    <row r="75" spans="1:135">
+    <row r="75" spans="1:138">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -11982,8 +12249,11 @@
       <c r="EC75" s="1"/>
       <c r="ED75" s="1"/>
       <c r="EE75" s="1"/>
+      <c r="EF75" s="1"/>
+      <c r="EG75" s="1"/>
+      <c r="EH75" s="1"/>
     </row>
-    <row r="76" spans="1:135">
+    <row r="76" spans="1:138">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -12119,8 +12389,11 @@
       <c r="EC76" s="1"/>
       <c r="ED76" s="1"/>
       <c r="EE76" s="1"/>
+      <c r="EF76" s="1"/>
+      <c r="EG76" s="1"/>
+      <c r="EH76" s="1"/>
     </row>
-    <row r="77" spans="1:135">
+    <row r="77" spans="1:138">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -12256,8 +12529,11 @@
       <c r="EC77" s="1"/>
       <c r="ED77" s="1"/>
       <c r="EE77" s="1"/>
+      <c r="EF77" s="1"/>
+      <c r="EG77" s="1"/>
+      <c r="EH77" s="1"/>
     </row>
-    <row r="78" spans="1:135">
+    <row r="78" spans="1:138">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -12393,8 +12669,11 @@
       <c r="EC78" s="1"/>
       <c r="ED78" s="1"/>
       <c r="EE78" s="1"/>
+      <c r="EF78" s="1"/>
+      <c r="EG78" s="1"/>
+      <c r="EH78" s="1"/>
     </row>
-    <row r="79" spans="1:135">
+    <row r="79" spans="1:138">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -12530,8 +12809,11 @@
       <c r="EC79" s="1"/>
       <c r="ED79" s="1"/>
       <c r="EE79" s="1"/>
+      <c r="EF79" s="1"/>
+      <c r="EG79" s="1"/>
+      <c r="EH79" s="1"/>
     </row>
-    <row r="80" spans="1:135">
+    <row r="80" spans="1:138">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -12667,8 +12949,11 @@
       <c r="EC80" s="1"/>
       <c r="ED80" s="1"/>
       <c r="EE80" s="1"/>
+      <c r="EF80" s="1"/>
+      <c r="EG80" s="1"/>
+      <c r="EH80" s="1"/>
     </row>
-    <row r="81" spans="1:135">
+    <row r="81" spans="1:138">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -12804,8 +13089,11 @@
       <c r="EC81" s="1"/>
       <c r="ED81" s="1"/>
       <c r="EE81" s="1"/>
+      <c r="EF81" s="1"/>
+      <c r="EG81" s="1"/>
+      <c r="EH81" s="1"/>
     </row>
-    <row r="82" spans="1:135">
+    <row r="82" spans="1:138">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -12941,8 +13229,11 @@
       <c r="EC82" s="1"/>
       <c r="ED82" s="1"/>
       <c r="EE82" s="1"/>
+      <c r="EF82" s="1"/>
+      <c r="EG82" s="1"/>
+      <c r="EH82" s="1"/>
     </row>
-    <row r="83" spans="1:135">
+    <row r="83" spans="1:138">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -13078,8 +13369,11 @@
       <c r="EC83" s="1"/>
       <c r="ED83" s="1"/>
       <c r="EE83" s="1"/>
+      <c r="EF83" s="1"/>
+      <c r="EG83" s="1"/>
+      <c r="EH83" s="1"/>
     </row>
-    <row r="84" spans="1:135">
+    <row r="84" spans="1:138">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -13215,8 +13509,11 @@
       <c r="EC84" s="1"/>
       <c r="ED84" s="1"/>
       <c r="EE84" s="1"/>
+      <c r="EF84" s="1"/>
+      <c r="EG84" s="1"/>
+      <c r="EH84" s="1"/>
     </row>
-    <row r="85" spans="1:135">
+    <row r="85" spans="1:138">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -13352,8 +13649,11 @@
       <c r="EC85" s="1"/>
       <c r="ED85" s="1"/>
       <c r="EE85" s="1"/>
+      <c r="EF85" s="1"/>
+      <c r="EG85" s="1"/>
+      <c r="EH85" s="1"/>
     </row>
-    <row r="86" spans="1:135">
+    <row r="86" spans="1:138">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -13489,8 +13789,11 @@
       <c r="EC86" s="1"/>
       <c r="ED86" s="1"/>
       <c r="EE86" s="1"/>
+      <c r="EF86" s="1"/>
+      <c r="EG86" s="1"/>
+      <c r="EH86" s="1"/>
     </row>
-    <row r="87" spans="1:135">
+    <row r="87" spans="1:138">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -13626,8 +13929,11 @@
       <c r="EC87" s="1"/>
       <c r="ED87" s="1"/>
       <c r="EE87" s="1"/>
+      <c r="EF87" s="1"/>
+      <c r="EG87" s="1"/>
+      <c r="EH87" s="1"/>
     </row>
-    <row r="88" spans="1:135">
+    <row r="88" spans="1:138">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -13763,8 +14069,11 @@
       <c r="EC88" s="1"/>
       <c r="ED88" s="1"/>
       <c r="EE88" s="1"/>
+      <c r="EF88" s="1"/>
+      <c r="EG88" s="1"/>
+      <c r="EH88" s="1"/>
     </row>
-    <row r="89" spans="1:135">
+    <row r="89" spans="1:138">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -13900,8 +14209,11 @@
       <c r="EC89" s="1"/>
       <c r="ED89" s="1"/>
       <c r="EE89" s="1"/>
+      <c r="EF89" s="1"/>
+      <c r="EG89" s="1"/>
+      <c r="EH89" s="1"/>
     </row>
-    <row r="90" spans="1:135">
+    <row r="90" spans="1:138">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -14037,8 +14349,11 @@
       <c r="EC90" s="1"/>
       <c r="ED90" s="1"/>
       <c r="EE90" s="1"/>
+      <c r="EF90" s="1"/>
+      <c r="EG90" s="1"/>
+      <c r="EH90" s="1"/>
     </row>
-    <row r="91" spans="1:135">
+    <row r="91" spans="1:138">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -14174,8 +14489,11 @@
       <c r="EC91" s="1"/>
       <c r="ED91" s="1"/>
       <c r="EE91" s="1"/>
+      <c r="EF91" s="1"/>
+      <c r="EG91" s="1"/>
+      <c r="EH91" s="1"/>
     </row>
-    <row r="92" spans="1:135">
+    <row r="92" spans="1:138">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -14311,8 +14629,11 @@
       <c r="EC92" s="1"/>
       <c r="ED92" s="1"/>
       <c r="EE92" s="1"/>
+      <c r="EF92" s="1"/>
+      <c r="EG92" s="1"/>
+      <c r="EH92" s="1"/>
     </row>
-    <row r="93" spans="1:135">
+    <row r="93" spans="1:138">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -14448,8 +14769,11 @@
       <c r="EC93" s="1"/>
       <c r="ED93" s="1"/>
       <c r="EE93" s="1"/>
+      <c r="EF93" s="1"/>
+      <c r="EG93" s="1"/>
+      <c r="EH93" s="1"/>
     </row>
-    <row r="94" spans="1:135">
+    <row r="94" spans="1:138">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -14585,8 +14909,11 @@
       <c r="EC94" s="1"/>
       <c r="ED94" s="1"/>
       <c r="EE94" s="1"/>
+      <c r="EF94" s="1"/>
+      <c r="EG94" s="1"/>
+      <c r="EH94" s="1"/>
     </row>
-    <row r="95" spans="1:135">
+    <row r="95" spans="1:138">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -14722,8 +15049,11 @@
       <c r="EC95" s="1"/>
       <c r="ED95" s="1"/>
       <c r="EE95" s="1"/>
+      <c r="EF95" s="1"/>
+      <c r="EG95" s="1"/>
+      <c r="EH95" s="1"/>
     </row>
-    <row r="96" spans="1:135">
+    <row r="96" spans="1:138">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -14859,8 +15189,11 @@
       <c r="EC96" s="1"/>
       <c r="ED96" s="1"/>
       <c r="EE96" s="1"/>
+      <c r="EF96" s="1"/>
+      <c r="EG96" s="1"/>
+      <c r="EH96" s="1"/>
     </row>
-    <row r="97" spans="1:135">
+    <row r="97" spans="1:138">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -14996,8 +15329,11 @@
       <c r="EC97" s="1"/>
       <c r="ED97" s="1"/>
       <c r="EE97" s="1"/>
+      <c r="EF97" s="1"/>
+      <c r="EG97" s="1"/>
+      <c r="EH97" s="1"/>
     </row>
-    <row r="98" spans="1:135">
+    <row r="98" spans="1:138">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -15133,8 +15469,11 @@
       <c r="EC98" s="1"/>
       <c r="ED98" s="1"/>
       <c r="EE98" s="1"/>
+      <c r="EF98" s="1"/>
+      <c r="EG98" s="1"/>
+      <c r="EH98" s="1"/>
     </row>
-    <row r="99" spans="1:135">
+    <row r="99" spans="1:138">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -15270,8 +15609,11 @@
       <c r="EC99" s="1"/>
       <c r="ED99" s="1"/>
       <c r="EE99" s="1"/>
+      <c r="EF99" s="1"/>
+      <c r="EG99" s="1"/>
+      <c r="EH99" s="1"/>
     </row>
-    <row r="100" spans="1:135">
+    <row r="100" spans="1:138">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -15407,8 +15749,11 @@
       <c r="EC100" s="1"/>
       <c r="ED100" s="1"/>
       <c r="EE100" s="1"/>
+      <c r="EF100" s="1"/>
+      <c r="EG100" s="1"/>
+      <c r="EH100" s="1"/>
     </row>
-    <row r="101" spans="1:135">
+    <row r="101" spans="1:138">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -15544,8 +15889,11 @@
       <c r="EC101" s="1"/>
       <c r="ED101" s="1"/>
       <c r="EE101" s="1"/>
+      <c r="EF101" s="1"/>
+      <c r="EG101" s="1"/>
+      <c r="EH101" s="1"/>
     </row>
-    <row r="102" spans="1:135">
+    <row r="102" spans="1:138">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -15681,8 +16029,11 @@
       <c r="EC102" s="1"/>
       <c r="ED102" s="1"/>
       <c r="EE102" s="1"/>
+      <c r="EF102" s="1"/>
+      <c r="EG102" s="1"/>
+      <c r="EH102" s="1"/>
     </row>
-    <row r="103" spans="1:135">
+    <row r="103" spans="1:138">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -15818,8 +16169,11 @@
       <c r="EC103" s="1"/>
       <c r="ED103" s="1"/>
       <c r="EE103" s="1"/>
+      <c r="EF103" s="1"/>
+      <c r="EG103" s="1"/>
+      <c r="EH103" s="1"/>
     </row>
-    <row r="104" spans="1:135">
+    <row r="104" spans="1:138">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -15955,8 +16309,11 @@
       <c r="EC104" s="1"/>
       <c r="ED104" s="1"/>
       <c r="EE104" s="1"/>
+      <c r="EF104" s="1"/>
+      <c r="EG104" s="1"/>
+      <c r="EH104" s="1"/>
     </row>
-    <row r="105" spans="1:135">
+    <row r="105" spans="1:138">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -16092,8 +16449,11 @@
       <c r="EC105" s="1"/>
       <c r="ED105" s="1"/>
       <c r="EE105" s="1"/>
+      <c r="EF105" s="1"/>
+      <c r="EG105" s="1"/>
+      <c r="EH105" s="1"/>
     </row>
-    <row r="106" spans="1:135">
+    <row r="106" spans="1:138">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -16229,8 +16589,11 @@
       <c r="EC106" s="1"/>
       <c r="ED106" s="1"/>
       <c r="EE106" s="1"/>
+      <c r="EF106" s="1"/>
+      <c r="EG106" s="1"/>
+      <c r="EH106" s="1"/>
     </row>
-    <row r="107" spans="1:135">
+    <row r="107" spans="1:138">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -16366,8 +16729,11 @@
       <c r="EC107" s="1"/>
       <c r="ED107" s="1"/>
       <c r="EE107" s="1"/>
+      <c r="EF107" s="1"/>
+      <c r="EG107" s="1"/>
+      <c r="EH107" s="1"/>
     </row>
-    <row r="108" spans="1:135">
+    <row r="108" spans="1:138">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -16503,8 +16869,11 @@
       <c r="EC108" s="1"/>
       <c r="ED108" s="1"/>
       <c r="EE108" s="1"/>
+      <c r="EF108" s="1"/>
+      <c r="EG108" s="1"/>
+      <c r="EH108" s="1"/>
     </row>
-    <row r="109" spans="1:135">
+    <row r="109" spans="1:138">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -16640,8 +17009,11 @@
       <c r="EC109" s="1"/>
       <c r="ED109" s="1"/>
       <c r="EE109" s="1"/>
+      <c r="EF109" s="1"/>
+      <c r="EG109" s="1"/>
+      <c r="EH109" s="1"/>
     </row>
-    <row r="110" spans="1:135">
+    <row r="110" spans="1:138">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -16777,8 +17149,11 @@
       <c r="EC110" s="1"/>
       <c r="ED110" s="1"/>
       <c r="EE110" s="1"/>
+      <c r="EF110" s="1"/>
+      <c r="EG110" s="1"/>
+      <c r="EH110" s="1"/>
     </row>
-    <row r="111" spans="1:135">
+    <row r="111" spans="1:138">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -16914,8 +17289,11 @@
       <c r="EC111" s="1"/>
       <c r="ED111" s="1"/>
       <c r="EE111" s="1"/>
+      <c r="EF111" s="1"/>
+      <c r="EG111" s="1"/>
+      <c r="EH111" s="1"/>
     </row>
-    <row r="112" spans="1:135">
+    <row r="112" spans="1:138">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -17051,8 +17429,11 @@
       <c r="EC112" s="1"/>
       <c r="ED112" s="1"/>
       <c r="EE112" s="1"/>
+      <c r="EF112" s="1"/>
+      <c r="EG112" s="1"/>
+      <c r="EH112" s="1"/>
     </row>
-    <row r="113" spans="1:135">
+    <row r="113" spans="1:138">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -17188,8 +17569,11 @@
       <c r="EC113" s="1"/>
       <c r="ED113" s="1"/>
       <c r="EE113" s="1"/>
+      <c r="EF113" s="1"/>
+      <c r="EG113" s="1"/>
+      <c r="EH113" s="1"/>
     </row>
-    <row r="114" spans="1:135">
+    <row r="114" spans="1:138">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -17325,8 +17709,11 @@
       <c r="EC114" s="1"/>
       <c r="ED114" s="1"/>
       <c r="EE114" s="1"/>
+      <c r="EF114" s="1"/>
+      <c r="EG114" s="1"/>
+      <c r="EH114" s="1"/>
     </row>
-    <row r="115" spans="1:135">
+    <row r="115" spans="1:138">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -17462,8 +17849,11 @@
       <c r="EC115" s="1"/>
       <c r="ED115" s="1"/>
       <c r="EE115" s="1"/>
+      <c r="EF115" s="1"/>
+      <c r="EG115" s="1"/>
+      <c r="EH115" s="1"/>
     </row>
-    <row r="116" spans="1:135">
+    <row r="116" spans="1:138">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -17599,8 +17989,11 @@
       <c r="EC116" s="1"/>
       <c r="ED116" s="1"/>
       <c r="EE116" s="1"/>
+      <c r="EF116" s="1"/>
+      <c r="EG116" s="1"/>
+      <c r="EH116" s="1"/>
     </row>
-    <row r="117" spans="1:135">
+    <row r="117" spans="1:138">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -17736,8 +18129,11 @@
       <c r="EC117" s="1"/>
       <c r="ED117" s="1"/>
       <c r="EE117" s="1"/>
+      <c r="EF117" s="1"/>
+      <c r="EG117" s="1"/>
+      <c r="EH117" s="1"/>
     </row>
-    <row r="118" spans="1:135">
+    <row r="118" spans="1:138">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -17873,8 +18269,11 @@
       <c r="EC118" s="1"/>
       <c r="ED118" s="1"/>
       <c r="EE118" s="1"/>
+      <c r="EF118" s="1"/>
+      <c r="EG118" s="1"/>
+      <c r="EH118" s="1"/>
     </row>
-    <row r="119" spans="1:135">
+    <row r="119" spans="1:138">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -18010,8 +18409,11 @@
       <c r="EC119" s="1"/>
       <c r="ED119" s="1"/>
       <c r="EE119" s="1"/>
+      <c r="EF119" s="1"/>
+      <c r="EG119" s="1"/>
+      <c r="EH119" s="1"/>
     </row>
-    <row r="120" spans="1:135">
+    <row r="120" spans="1:138">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -18147,8 +18549,11 @@
       <c r="EC120" s="1"/>
       <c r="ED120" s="1"/>
       <c r="EE120" s="1"/>
+      <c r="EF120" s="1"/>
+      <c r="EG120" s="1"/>
+      <c r="EH120" s="1"/>
     </row>
-    <row r="121" spans="1:135">
+    <row r="121" spans="1:138">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -18284,8 +18689,11 @@
       <c r="EC121" s="1"/>
       <c r="ED121" s="1"/>
       <c r="EE121" s="1"/>
+      <c r="EF121" s="1"/>
+      <c r="EG121" s="1"/>
+      <c r="EH121" s="1"/>
     </row>
-    <row r="122" spans="1:135">
+    <row r="122" spans="1:138">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -18421,8 +18829,11 @@
       <c r="EC122" s="1"/>
       <c r="ED122" s="1"/>
       <c r="EE122" s="1"/>
+      <c r="EF122" s="1"/>
+      <c r="EG122" s="1"/>
+      <c r="EH122" s="1"/>
     </row>
-    <row r="123" spans="1:135">
+    <row r="123" spans="1:138">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -18558,8 +18969,11 @@
       <c r="EC123" s="1"/>
       <c r="ED123" s="1"/>
       <c r="EE123" s="1"/>
+      <c r="EF123" s="1"/>
+      <c r="EG123" s="1"/>
+      <c r="EH123" s="1"/>
     </row>
-    <row r="124" spans="1:135">
+    <row r="124" spans="1:138">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -18695,8 +19109,11 @@
       <c r="EC124" s="1"/>
       <c r="ED124" s="1"/>
       <c r="EE124" s="1"/>
+      <c r="EF124" s="1"/>
+      <c r="EG124" s="1"/>
+      <c r="EH124" s="1"/>
     </row>
-    <row r="125" spans="1:135">
+    <row r="125" spans="1:138">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -18832,8 +19249,11 @@
       <c r="EC125" s="1"/>
       <c r="ED125" s="1"/>
       <c r="EE125" s="1"/>
+      <c r="EF125" s="1"/>
+      <c r="EG125" s="1"/>
+      <c r="EH125" s="1"/>
     </row>
-    <row r="126" spans="1:135">
+    <row r="126" spans="1:138">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -18969,8 +19389,11 @@
       <c r="EC126" s="1"/>
       <c r="ED126" s="1"/>
       <c r="EE126" s="1"/>
+      <c r="EF126" s="1"/>
+      <c r="EG126" s="1"/>
+      <c r="EH126" s="1"/>
     </row>
-    <row r="127" spans="1:135">
+    <row r="127" spans="1:138">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -19106,8 +19529,11 @@
       <c r="EC127" s="1"/>
       <c r="ED127" s="1"/>
       <c r="EE127" s="1"/>
+      <c r="EF127" s="1"/>
+      <c r="EG127" s="1"/>
+      <c r="EH127" s="1"/>
     </row>
-    <row r="128" spans="1:135">
+    <row r="128" spans="1:138">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -19243,8 +19669,11 @@
       <c r="EC128" s="1"/>
       <c r="ED128" s="1"/>
       <c r="EE128" s="1"/>
+      <c r="EF128" s="1"/>
+      <c r="EG128" s="1"/>
+      <c r="EH128" s="1"/>
     </row>
-    <row r="129" spans="1:135">
+    <row r="129" spans="1:138">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -19380,8 +19809,11 @@
       <c r="EC129" s="1"/>
       <c r="ED129" s="1"/>
       <c r="EE129" s="1"/>
+      <c r="EF129" s="1"/>
+      <c r="EG129" s="1"/>
+      <c r="EH129" s="1"/>
     </row>
-    <row r="130" spans="1:135">
+    <row r="130" spans="1:138">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -19517,8 +19949,11 @@
       <c r="EC130" s="1"/>
       <c r="ED130" s="1"/>
       <c r="EE130" s="1"/>
+      <c r="EF130" s="1"/>
+      <c r="EG130" s="1"/>
+      <c r="EH130" s="1"/>
     </row>
-    <row r="131" spans="1:135">
+    <row r="131" spans="1:138">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -19654,8 +20089,11 @@
       <c r="EC131" s="1"/>
       <c r="ED131" s="1"/>
       <c r="EE131" s="1"/>
+      <c r="EF131" s="1"/>
+      <c r="EG131" s="1"/>
+      <c r="EH131" s="1"/>
     </row>
-    <row r="132" spans="1:135">
+    <row r="132" spans="1:138">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -19791,8 +20229,11 @@
       <c r="EC132" s="1"/>
       <c r="ED132" s="1"/>
       <c r="EE132" s="1"/>
+      <c r="EF132" s="1"/>
+      <c r="EG132" s="1"/>
+      <c r="EH132" s="1"/>
     </row>
-    <row r="133" spans="1:135">
+    <row r="133" spans="1:138">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -19928,8 +20369,11 @@
       <c r="EC133" s="1"/>
       <c r="ED133" s="1"/>
       <c r="EE133" s="1"/>
+      <c r="EF133" s="1"/>
+      <c r="EG133" s="1"/>
+      <c r="EH133" s="1"/>
     </row>
-    <row r="134" spans="1:135">
+    <row r="134" spans="1:138">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -20065,8 +20509,11 @@
       <c r="EC134" s="1"/>
       <c r="ED134" s="1"/>
       <c r="EE134" s="1"/>
+      <c r="EF134" s="1"/>
+      <c r="EG134" s="1"/>
+      <c r="EH134" s="1"/>
     </row>
-    <row r="135" spans="1:135">
+    <row r="135" spans="1:138">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -20202,8 +20649,11 @@
       <c r="EC135" s="1"/>
       <c r="ED135" s="1"/>
       <c r="EE135" s="1"/>
+      <c r="EF135" s="1"/>
+      <c r="EG135" s="1"/>
+      <c r="EH135" s="1"/>
     </row>
-    <row r="136" spans="1:135">
+    <row r="136" spans="1:138">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -20339,8 +20789,11 @@
       <c r="EC136" s="1"/>
       <c r="ED136" s="1"/>
       <c r="EE136" s="1"/>
+      <c r="EF136" s="1"/>
+      <c r="EG136" s="1"/>
+      <c r="EH136" s="1"/>
     </row>
-    <row r="137" spans="1:135">
+    <row r="137" spans="1:138">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -20476,8 +20929,11 @@
       <c r="EC137" s="1"/>
       <c r="ED137" s="1"/>
       <c r="EE137" s="1"/>
+      <c r="EF137" s="1"/>
+      <c r="EG137" s="1"/>
+      <c r="EH137" s="1"/>
     </row>
-    <row r="138" spans="1:135">
+    <row r="138" spans="1:138">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -20613,8 +21069,11 @@
       <c r="EC138" s="1"/>
       <c r="ED138" s="1"/>
       <c r="EE138" s="1"/>
+      <c r="EF138" s="1"/>
+      <c r="EG138" s="1"/>
+      <c r="EH138" s="1"/>
     </row>
-    <row r="139" spans="1:135">
+    <row r="139" spans="1:138">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -20750,8 +21209,11 @@
       <c r="EC139" s="1"/>
       <c r="ED139" s="1"/>
       <c r="EE139" s="1"/>
+      <c r="EF139" s="1"/>
+      <c r="EG139" s="1"/>
+      <c r="EH139" s="1"/>
     </row>
-    <row r="140" spans="1:135">
+    <row r="140" spans="1:138">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -20887,8 +21349,11 @@
       <c r="EC140" s="1"/>
       <c r="ED140" s="1"/>
       <c r="EE140" s="1"/>
+      <c r="EF140" s="1"/>
+      <c r="EG140" s="1"/>
+      <c r="EH140" s="1"/>
     </row>
-    <row r="141" spans="1:135">
+    <row r="141" spans="1:138">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -21024,8 +21489,11 @@
       <c r="EC141" s="1"/>
       <c r="ED141" s="1"/>
       <c r="EE141" s="1"/>
+      <c r="EF141" s="1"/>
+      <c r="EG141" s="1"/>
+      <c r="EH141" s="1"/>
     </row>
-    <row r="142" spans="1:135">
+    <row r="142" spans="1:138">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -21161,8 +21629,11 @@
       <c r="EC142" s="1"/>
       <c r="ED142" s="1"/>
       <c r="EE142" s="1"/>
+      <c r="EF142" s="1"/>
+      <c r="EG142" s="1"/>
+      <c r="EH142" s="1"/>
     </row>
-    <row r="143" spans="1:135">
+    <row r="143" spans="1:138">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -21298,8 +21769,11 @@
       <c r="EC143" s="1"/>
       <c r="ED143" s="1"/>
       <c r="EE143" s="1"/>
+      <c r="EF143" s="1"/>
+      <c r="EG143" s="1"/>
+      <c r="EH143" s="1"/>
     </row>
-    <row r="144" spans="1:135">
+    <row r="144" spans="1:138">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -21435,8 +21909,11 @@
       <c r="EC144" s="1"/>
       <c r="ED144" s="1"/>
       <c r="EE144" s="1"/>
+      <c r="EF144" s="1"/>
+      <c r="EG144" s="1"/>
+      <c r="EH144" s="1"/>
     </row>
-    <row r="145" spans="1:135">
+    <row r="145" spans="1:138">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -21572,8 +22049,11 @@
       <c r="EC145" s="1"/>
       <c r="ED145" s="1"/>
       <c r="EE145" s="1"/>
+      <c r="EF145" s="1"/>
+      <c r="EG145" s="1"/>
+      <c r="EH145" s="1"/>
     </row>
-    <row r="146" spans="1:135">
+    <row r="146" spans="1:138">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -21709,8 +22189,11 @@
       <c r="EC146" s="1"/>
       <c r="ED146" s="1"/>
       <c r="EE146" s="1"/>
+      <c r="EF146" s="1"/>
+      <c r="EG146" s="1"/>
+      <c r="EH146" s="1"/>
     </row>
-    <row r="147" spans="1:135">
+    <row r="147" spans="1:138">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -21846,8 +22329,11 @@
       <c r="EC147" s="1"/>
       <c r="ED147" s="1"/>
       <c r="EE147" s="1"/>
+      <c r="EF147" s="1"/>
+      <c r="EG147" s="1"/>
+      <c r="EH147" s="1"/>
     </row>
-    <row r="148" spans="1:135">
+    <row r="148" spans="1:138">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -21983,8 +22469,11 @@
       <c r="EC148" s="1"/>
       <c r="ED148" s="1"/>
       <c r="EE148" s="1"/>
+      <c r="EF148" s="1"/>
+      <c r="EG148" s="1"/>
+      <c r="EH148" s="1"/>
     </row>
-    <row r="149" spans="1:135">
+    <row r="149" spans="1:138">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -22120,8 +22609,11 @@
       <c r="EC149" s="1"/>
       <c r="ED149" s="1"/>
       <c r="EE149" s="1"/>
+      <c r="EF149" s="1"/>
+      <c r="EG149" s="1"/>
+      <c r="EH149" s="1"/>
     </row>
-    <row r="150" spans="1:135">
+    <row r="150" spans="1:138">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -22257,8 +22749,11 @@
       <c r="EC150" s="1"/>
       <c r="ED150" s="1"/>
       <c r="EE150" s="1"/>
+      <c r="EF150" s="1"/>
+      <c r="EG150" s="1"/>
+      <c r="EH150" s="1"/>
     </row>
-    <row r="151" spans="1:135">
+    <row r="151" spans="1:138">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -22394,8 +22889,11 @@
       <c r="EC151" s="1"/>
       <c r="ED151" s="1"/>
       <c r="EE151" s="1"/>
+      <c r="EF151" s="1"/>
+      <c r="EG151" s="1"/>
+      <c r="EH151" s="1"/>
     </row>
-    <row r="152" spans="1:135">
+    <row r="152" spans="1:138">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -22531,8 +23029,11 @@
       <c r="EC152" s="1"/>
       <c r="ED152" s="1"/>
       <c r="EE152" s="1"/>
+      <c r="EF152" s="1"/>
+      <c r="EG152" s="1"/>
+      <c r="EH152" s="1"/>
     </row>
-    <row r="153" spans="1:135">
+    <row r="153" spans="1:138">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -22668,8 +23169,11 @@
       <c r="EC153" s="1"/>
       <c r="ED153" s="1"/>
       <c r="EE153" s="1"/>
+      <c r="EF153" s="1"/>
+      <c r="EG153" s="1"/>
+      <c r="EH153" s="1"/>
     </row>
-    <row r="154" spans="1:135">
+    <row r="154" spans="1:138">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -22805,6 +23309,9 @@
       <c r="EC154" s="1"/>
       <c r="ED154" s="1"/>
       <c r="EE154" s="1"/>
+      <c r="EF154" s="1"/>
+      <c r="EG154" s="1"/>
+      <c r="EH154" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>